<commit_message>
approved commit and good stuff.
</commit_message>
<xml_diff>
--- a/audit/docker_benchmark_reports/192.168.1.8_section1.xlsx
+++ b/audit/docker_benchmark_reports/192.168.1.8_section1.xlsx
@@ -876,7 +876,7 @@
     <row r="4" ht="16" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Host: Docker-2204-DA-AUTO   |   OS: Ubuntu 22.04   |   Generated: 2026-05-18T05:56:21Z</t>
+          <t>Host: Docker-2204-DA-AUTO   |   OS: Ubuntu 22.04   |   Generated: 2026-05-21T18:48:40Z</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="J14" s="15" t="inlineStr">
         <is>
-          <t>[INFO] 1.1.2 - Manual review required. Docker group members: docker:x:999:</t>
+          <t>[INFO] 1.1.2 - Manual review required. Docker group members: docker:x:999:v1nh2oz4</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="F3" s="12" t="inlineStr">
         <is>
-          <t>[INFO] 1.1.2 - Manual review required. Docker group members: docker:x:999:</t>
+          <t>[INFO] 1.1.2 - Manual review required. Docker group members: docker:x:999:v1nh2oz4</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
     <row r="5" ht="14" customHeight="1">
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "generated": "2026-05-18T05:56:21Z",</t>
+          <t xml:space="preserve">    "generated": "2026-05-21T18:48:40Z",</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2252,7 @@
     <row r="21" ht="14" customHeight="1">
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "details": "[INFO] 1.1.2 - Manual review required. Docker group members: docker:x:999:",</t>
+          <t xml:space="preserve">      "details": "[INFO] 1.1.2 - Manual review required. Docker group members: docker:x:999:v1nh2oz4",</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix repeeting json file.
</commit_message>
<xml_diff>
--- a/audit/docker_benchmark_reports/192.168.1.8_section1.xlsx
+++ b/audit/docker_benchmark_reports/192.168.1.8_section1.xlsx
@@ -876,7 +876,7 @@
     <row r="4" ht="16" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Host: Docker-2204-DA-AUTO   |   OS: Ubuntu 22.04   |   Generated: 2026-05-21T18:48:40Z</t>
+          <t>Host: Docker-2204-DA-AUTO   |   OS: Ubuntu 22.04   |   Generated: 2026-05-28T13:03:46Z</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
     <row r="5" ht="14" customHeight="1">
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "generated": "2026-05-21T18:48:40Z",</t>
+          <t xml:space="preserve">    "generated": "2026-05-28T13:03:46Z",</t>
         </is>
       </c>
     </row>

</xml_diff>